<commit_message>
Tabela com dados atualizados
</commit_message>
<xml_diff>
--- a/dados_modelo.xlsx
+++ b/dados_modelo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROGRAMMING\MACHINE LEARNING\API_MODELO_IA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37CED823-B2EA-4C5C-90FF-395A6095058C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{302DC8A4-B75B-4677-8A27-D36986B8E3B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5715" yWindow="3885" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -387,10 +387,10 @@
         <v>18</v>
       </c>
       <c r="B2">
-        <v>1200</v>
+        <v>5500</v>
       </c>
       <c r="C2">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -409,10 +409,10 @@
         <v>25</v>
       </c>
       <c r="B4">
-        <v>2500</v>
+        <v>4000</v>
       </c>
       <c r="C4">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -461,10 +461,10 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="B9">
-        <v>6500</v>
+        <v>6000</v>
       </c>
       <c r="C9">
         <v>1</v>
@@ -472,24 +472,24 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="B10">
-        <v>7200</v>
+        <v>6300</v>
       </c>
       <c r="C10">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="B11">
-        <v>8000</v>
+        <v>7000</v>
       </c>
       <c r="C11">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>